<commit_message>
Dynamic and robust logic for all platform sections
Implemented a dynamic, robust, and generic logic to avoid code repetition across all platform sections.

The front-end implementation is largely complete, ensuring scalability and maintainability.

Remaining tasks include adding features such as file uploads to define models within each scenario.
</commit_message>
<xml_diff>
--- a/backend/{templates}/financial-statements-{model}.xlsx
+++ b/backend/{templates}/financial-statements-{model}.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8954da175e61d5af/Escritorio/IIT/CC-WBT/backend/{templates}/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="555" documentId="10_ncr:20000_{4F2B366B-AA2F-4F18-863E-957538EF6F0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{74257CA7-F20E-40C0-821E-E093AE44EDF2}"/>
+  <xr:revisionPtr revIDLastSave="558" documentId="10_ncr:20000_{4F2B366B-AA2F-4F18-863E-957538EF6F0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A84C2DA7-BAC2-46F8-9F9B-D92693233714}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="E-Cooking" sheetId="2" r:id="rId1"/>
-    <sheet name="Electricity" sheetId="6" r:id="rId2"/>
-    <sheet name="Electricity (Low access)" sheetId="5" r:id="rId3"/>
+    <sheet name="Electricity (Only E-Cooking)" sheetId="2" r:id="rId1"/>
+    <sheet name="Electricity &amp; E-Cooking" sheetId="6" r:id="rId2"/>
+    <sheet name="Electricity (Just access)" sheetId="5" r:id="rId3"/>
     <sheet name="LPG" sheetId="1" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029" iterate="1"/>

</xml_diff>